<commit_message>
iterative opponent-weighted ratings, validation jumped from 42% to 92% winner accuracy
</commit_message>
<xml_diff>
--- a/inputs/manual_adjustments.xlsx
+++ b/inputs/manual_adjustments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6313b40ac91b0b3d/Desktop/PersonalProjects/worldcup-sim/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="11_F25DC773A252ABDACC10488DB19F67AA5BDE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4F62531-F32A-4A48-B08B-1A1D99CFE6BB}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="11_F25DC773A252ABDACC10488DB19F67AA5BDE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02919080-58EB-4BD9-90E8-58522EE7603E}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13785" yWindow="795" windowWidth="15015" windowHeight="14385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1311,10 +1311,10 @@
         <v>-0.1</v>
       </c>
       <c r="C41" s="2">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="D41" s="2">
-        <v>-0.05</v>
+        <v>-0.01</v>
       </c>
       <c r="E41" s="2">
         <v>0</v>

</xml_diff>